<commit_message>
CoPo auswertung fertig und werte angepasst
</commit_message>
<xml_diff>
--- a/Copolymerisation/Messwerte/Messwerte-und-Auswertung.xlsx
+++ b/Copolymerisation/Messwerte/Messwerte-und-Auswertung.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dokumente\Uni laptop\Chemie\Poly\Copolymerisation\Messwerte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDA452A-142C-40BD-B872-0855A03F53B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCEF825-C52D-47D9-AEC2-1C11E57B0EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9015" yWindow="1050" windowWidth="18720" windowHeight="14325" xr2:uid="{EC9A12D4-FC17-4DF3-91C2-7490D74CCC1E}"/>
+    <workbookView xWindow="2040" yWindow="1455" windowWidth="19410" windowHeight="13905" xr2:uid="{EC9A12D4-FC17-4DF3-91C2-7490D74CCC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>Probe</t>
   </si>
@@ -114,6 +114,12 @@
   </si>
   <si>
     <t>n_St^2/n_MMA^2 * 1/(m_St/m_MMA)</t>
+  </si>
+  <si>
+    <t>n_St/(n_St+n_MMA)</t>
+  </si>
+  <si>
+    <t>m_St/(m_St+m_MMA</t>
   </si>
 </sst>
 </file>
@@ -486,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E9289F-E3E9-4E4D-BE1F-9BBD6364599B}">
-  <dimension ref="B2:L44"/>
+  <dimension ref="B2:L53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -669,12 +675,12 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <f>0.9*2</f>
-        <v>1.8</v>
+        <f>G13*$B$24/5</f>
+        <v>20.830000000000002</v>
       </c>
       <c r="F13">
-        <f>0.94*10</f>
-        <v>9.3999999999999986</v>
+        <f>H13*$B$26/3</f>
+        <v>85.770323333333337</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -688,15 +694,15 @@
       </c>
       <c r="J13">
         <f>E13/$B$24</f>
-        <v>1.728276524243879E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K13">
         <f>F13/$B$26</f>
-        <v>9.3886397459074511E-2</v>
+        <v>0.8566666666666668</v>
       </c>
       <c r="L13">
         <f>J13/K13</f>
-        <v>0.18408167434449088</v>
+        <v>0.23346303501945523</v>
       </c>
     </row>
     <row r="14" spans="4:12" x14ac:dyDescent="0.25">
@@ -704,12 +710,12 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <f>0.9*4</f>
-        <v>3.6</v>
+        <f t="shared" ref="E14:E17" si="6">G14*$B$24/5</f>
+        <v>20.830000000000002</v>
       </c>
       <c r="F14">
-        <f>0.94*8</f>
-        <v>7.52</v>
+        <f t="shared" ref="F14:F17" si="7">H14*$B$26/3</f>
+        <v>32.038719999999998</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -718,20 +724,20 @@
         <v>0.96</v>
       </c>
       <c r="I14">
-        <f t="shared" ref="I14:I17" si="6">(G14/H14)*($B$24/$B$26)*(3/5)</f>
+        <f t="shared" ref="I14:I17" si="8">(G14/H14)*($B$24/$B$26)*(3/5)</f>
         <v>0.65015081751081194</v>
       </c>
       <c r="J14">
         <f>E14/$B$24</f>
-        <v>3.456553048487758E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K14">
         <f>F14/$B$26</f>
-        <v>7.5109117967259609E-2</v>
+        <v>0.32</v>
       </c>
       <c r="L14">
-        <f t="shared" ref="L14:L17" si="7">J14/K14</f>
-        <v>0.46020418586122719</v>
+        <f t="shared" ref="L14:L17" si="9">J14/K14</f>
+        <v>0.625</v>
       </c>
     </row>
     <row r="15" spans="4:12" x14ac:dyDescent="0.25">
@@ -739,12 +745,12 @@
         <v>3</v>
       </c>
       <c r="E15">
-        <f>0.9*6</f>
-        <v>5.4</v>
+        <f t="shared" si="6"/>
+        <v>20.830000000000002</v>
       </c>
       <c r="F15">
-        <f>0.94*6</f>
-        <v>5.64</v>
+        <f t="shared" si="7"/>
+        <v>14.016939999999998</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -753,20 +759,20 @@
         <v>0.42</v>
       </c>
       <c r="I15">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>1.4860590114532846</v>
       </c>
       <c r="J15">
         <f>E15/$B$24</f>
-        <v>5.1848295727316369E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K15">
         <f>F15/$B$26</f>
-        <v>5.6331838475444714E-2</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="L15">
-        <f t="shared" si="7"/>
-        <v>0.92040837172245427</v>
+        <f t="shared" si="9"/>
+        <v>1.4285714285714288</v>
       </c>
     </row>
     <row r="16" spans="4:12" x14ac:dyDescent="0.25">
@@ -774,12 +780,12 @@
         <v>4</v>
       </c>
       <c r="E16">
-        <f>0.9*8</f>
-        <v>7.2</v>
+        <f t="shared" si="6"/>
+        <v>20.830000000000002</v>
       </c>
       <c r="F16">
-        <f>0.94*4</f>
-        <v>3.76</v>
+        <f t="shared" si="7"/>
+        <v>9.3446266666666666</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -788,20 +794,20 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="I16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>2.2290885171799264</v>
       </c>
       <c r="J16">
         <f>E16/$B$24</f>
-        <v>6.9131060969755159E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K16">
         <f>F16/$B$26</f>
-        <v>3.7554558983629804E-2</v>
+        <v>9.3333333333333338E-2</v>
       </c>
       <c r="L16">
-        <f t="shared" si="7"/>
-        <v>1.8408167434449088</v>
+        <f t="shared" si="9"/>
+        <v>2.1428571428571428</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
@@ -809,12 +815,12 @@
         <v>5</v>
       </c>
       <c r="E17">
-        <f>0.9*10</f>
-        <v>9</v>
+        <f t="shared" si="6"/>
+        <v>20.830000000000002</v>
       </c>
       <c r="F17">
-        <f>0.94*2</f>
-        <v>1.88</v>
+        <f t="shared" si="7"/>
+        <v>5.0060499999999992</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -823,20 +829,20 @@
         <v>0.15</v>
       </c>
       <c r="I17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>4.1609652320691968</v>
       </c>
       <c r="J17">
         <f>E17/$B$24</f>
-        <v>8.6413826212193942E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K17">
         <f>F17/$B$26</f>
-        <v>1.8777279491814902E-2</v>
+        <v>4.9999999999999996E-2</v>
       </c>
       <c r="L17">
-        <f t="shared" si="7"/>
-        <v>4.6020418586122718</v>
+        <f t="shared" si="9"/>
+        <v>4.0000000000000009</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
@@ -894,7 +900,7 @@
         <v>0.96</v>
       </c>
       <c r="G22">
-        <f t="shared" ref="G22:G25" si="8">(E22/F22)*($B$24/$B$26)*(3/5)</f>
+        <f t="shared" ref="G22:G25" si="10">(E22/F22)*($B$24/$B$26)*(3/5)</f>
         <v>0.65015081751081194</v>
       </c>
       <c r="H22">
@@ -915,7 +921,7 @@
         <v>0.42</v>
       </c>
       <c r="G23">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.4860590114532846</v>
       </c>
       <c r="H23">
@@ -936,7 +942,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="G24">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>2.2290885171799264</v>
       </c>
       <c r="H24">
@@ -957,7 +963,7 @@
         <v>0.15</v>
       </c>
       <c r="G25">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>4.1609652320691968</v>
       </c>
       <c r="H25">
@@ -990,51 +996,51 @@
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32">
         <f>I13*((K13)^2/(J13)^2)</f>
-        <v>7.1668961408850862</v>
+        <v>4.455700269340765</v>
       </c>
       <c r="C32">
         <f>L13*(I13-1)</f>
-        <v>-0.1393759867875739</v>
+        <v>-0.17676469425937899</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f>I14*((K14)^2/(J14)^2)</f>
-        <v>3.0698205136791117</v>
+        <v>1.6643860928276784</v>
       </c>
       <c r="C33">
-        <f t="shared" ref="C33:C36" si="9">L14*(I14-1)</f>
-        <v>-0.1610020582016527</v>
+        <f t="shared" ref="C33:C36" si="11">L14*(I14-1)</f>
+        <v>-0.21865573905574254</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f>I15*((K15)^2/(J15)^2)</f>
-        <v>1.7541831506737788</v>
+        <v>0.72816891561210917</v>
       </c>
       <c r="C34">
-        <f t="shared" si="9"/>
-        <v>0.44737278329274338</v>
+        <f t="shared" si="11"/>
+        <v>0.69437001636183526</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f>I16*((K16)^2/(J16)^2)</f>
-        <v>0.65781868150266665</v>
+        <v>0.48544594374140615</v>
       </c>
       <c r="C35">
-        <f t="shared" si="9"/>
-        <v>2.2625267216006839</v>
+        <f t="shared" si="11"/>
+        <v>2.6337611082426995</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f>I17*((K17)^2/(J17)^2)</f>
-        <v>0.19646851287546321</v>
+        <v>0.26006032700432469</v>
       </c>
       <c r="C36">
-        <f t="shared" si="9"/>
-        <v>14.546894311600497</v>
+        <f t="shared" si="11"/>
+        <v>12.643860928276791</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
@@ -1048,51 +1054,109 @@
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f>J13/K13*(1-(1/I13))</f>
-        <v>-0.57389934957621735</v>
+        <v>-0.72785237544621906</v>
       </c>
       <c r="C40">
         <f>((J13)^2/(K13)^2)*(1/I13)</f>
-        <v>0.13953041600467556</v>
+        <v>0.22443161333828973</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
-        <f t="shared" ref="B41:B44" si="10">J14/K14*(1-(1/I14))</f>
-        <v>-0.24763801546550426</v>
+        <f t="shared" ref="B41:B44" si="12">J14/K14*(1-(1/I14))</f>
+        <v>-0.33631541046567448</v>
       </c>
       <c r="C41">
-        <f t="shared" ref="C41:C44" si="11">((J14)^2/(K14)^2)*(1/I14)</f>
-        <v>0.32575194397978735</v>
+        <f t="shared" ref="C41:C44" si="13">((J14)^2/(K14)^2)*(1/I14)</f>
+        <v>0.60082213154104658</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
-        <f t="shared" si="10"/>
-        <v>0.3010464455615644</v>
+        <f t="shared" si="12"/>
+        <v>0.46725601810575429</v>
       </c>
       <c r="C42">
-        <f t="shared" si="11"/>
-        <v>0.57006590196462759</v>
+        <f t="shared" si="13"/>
+        <v>1.3733077292366782</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
-        <f t="shared" si="10"/>
-        <v>1.0150008418970553</v>
+        <f t="shared" si="12"/>
+        <v>1.1815417323914683</v>
       </c>
       <c r="C43">
-        <f t="shared" si="11"/>
-        <v>1.5201757385723411</v>
+        <f t="shared" si="13"/>
+        <v>2.0599615938550171</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
-        <f t="shared" si="10"/>
-        <v>3.4960384190392539</v>
+        <f t="shared" si="12"/>
+        <v>3.0386845895343266</v>
       </c>
       <c r="C44">
-        <f t="shared" si="11"/>
-        <v>5.089874124684175</v>
+        <f t="shared" si="13"/>
+        <v>3.8452616418626993</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>26</v>
+      </c>
+      <c r="C48" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <f>J13/(J13+K13)</f>
+        <v>0.18927444794952678</v>
+      </c>
+      <c r="C49">
+        <f>E13/(E13+F13)</f>
+        <v>0.19540278442557571</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <f t="shared" ref="B50:B53" si="14">J14/(J14+K14)</f>
+        <v>0.38461538461538464</v>
+      </c>
+      <c r="C50">
+        <f t="shared" ref="C50:C53" si="15">E14/(E14+F14)</f>
+        <v>0.3939947855745326</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <f t="shared" si="14"/>
+        <v>0.58823529411764719</v>
+      </c>
+      <c r="C51">
+        <f t="shared" si="15"/>
+        <v>0.59775693360736981</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <f t="shared" si="14"/>
+        <v>0.68181818181818188</v>
+      </c>
+      <c r="C52">
+        <f t="shared" si="15"/>
+        <v>0.69031508591987001</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <f>J17/(J17+K17)</f>
+        <v>0.8</v>
+      </c>
+      <c r="C53">
+        <f t="shared" si="15"/>
+        <v>0.80623779563826525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>